<commit_message>
Selenium TestNG - TestNG Data Provider.
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -4,6 +4,10 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="demo" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="loginData" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="customers" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="products" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="Sheet4" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="41">
   <si>
     <t>name</t>
   </si>
@@ -47,13 +51,119 @@
   </si>
   <si>
     <t>selenium</t>
+  </si>
+  <si>
+    <t>userId</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>mngr643764</t>
+  </si>
+  <si>
+    <t>INVALIDPASS</t>
+  </si>
+  <si>
+    <t>INVALIDUSER</t>
+  </si>
+  <si>
+    <t>ujuturE</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>precilla</t>
+  </si>
+  <si>
+    <t>des</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>custID</t>
+  </si>
+  <si>
+    <t>macbook</t>
+  </si>
+  <si>
+    <t>macbook air</t>
+  </si>
+  <si>
+    <t>iphone</t>
+  </si>
+  <si>
+    <t>ihone 16</t>
+  </si>
+  <si>
+    <t>lenovo</t>
+  </si>
+  <si>
+    <t>lenovo yoga</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Effort (Days)</t>
+  </si>
+  <si>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Phase 1 - Mobilization</t>
+  </si>
+  <si>
+    <t>Considering Ready to Upload Data is available in standard format (CSV / JSON) from third party app</t>
+  </si>
+  <si>
+    <t>Phase 2 - EDP Training Dashboard</t>
+  </si>
+  <si>
+    <t>Considering Data is available to plot the required charts and graphs into the dashboard</t>
+  </si>
+  <si>
+    <t>Phase 3 - Sector Training and market
+linkages</t>
+  </si>
+  <si>
+    <t>TBD - Open for further discussion as this requires detailed overview of business flow.</t>
+  </si>
+  <si>
+    <t>Phase 4 - Demo day &amp; Funds</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">*Note* </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t>: 
+- Efforts are provided by having basline SRS document and Proofs documented provided earlier.
+- Each phase before beginning will require detailed demo and feedback reconciliation before commencement.
+- Deviations from provided timelines might occur in case of midway requirement revisions or significant deviations from assumptions
+- Efforts are calculated on basis of working days and NOT calendar days.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -65,22 +175,48 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF073763"/>
+        <bgColor rgb="FF073763"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -90,6 +226,16 @@
     <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -99,6 +245,22 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -351,4 +513,263 @@
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>3.80213821E8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1">
+        <v>8.13082193E9</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="1">
+        <v>999.0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="1">
+        <v>599.0</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="1">
+        <v>799.0</v>
+      </c>
+      <c r="D4" s="1">
+        <v>2.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="28.75"/>
+    <col customWidth="1" min="3" max="3" width="75.13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="4">
+        <v>20.0</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="6">
+        <f>SUM(B2:B5)</f>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>